<commit_message>
Separate operation date and value date for imports
- Make Value Date mandatory for transaction imports (with "Same as
  operation date" checkbox for single-date files)
- Auto-map: Data_Operazione -> date, Data_Valuta -> valueDate
- Wipe-and-replace uses operation date for cutoff (fixes wrong balance
  when re-importing with different date ranges)
- Date fallback: if operation date unparsable, use value date (and
  vice versa). Skip row only if both are unparsable.
- Add valueDate column to asset_events and incomes tables (DB v24)
- Localized field labels: Operation Date / Value Date
- Fix macOS deployment target warnings (Podfile post_install)
- Split import_flow_test.dart into 4 files (transaction, asset,
  income, dedup) for targeted re-execution
- 3 new unit tests for date fallback logic
</commit_message>
<xml_diff>
--- a/integration_test/fixtures/transactions_formula.xlsx
+++ b/integration_test/fixtures/transactions_formula.xlsx
@@ -11,9 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t xml:space="preserve">Date</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+  <si>
+    <t xml:space="preserve">Data_Operazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data_Valuta</t>
   </si>
   <si>
     <t xml:space="preserve">Debit</t>
@@ -293,47 +296,59 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2">
         <v>45698.0</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
+        <v>45698.0</v>
+      </c>
+      <c r="C2" s="3">
         <v>0.0</v>
       </c>
-      <c r="C2" s="3">
+      <c r="D2" s="3">
         <v>2000.0</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>4</v>
+      <c r="E2" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2">
         <v>45700.0</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
+        <v>45700.0</v>
+      </c>
+      <c r="C3" s="3">
         <v>150.0</v>
       </c>
-      <c r="C3" s="3">
+      <c r="D3" s="3">
         <v>0.0</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>5</v>
+      <c r="E3" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2">
         <v>45703.0</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
+        <v>45703.0</v>
+      </c>
+      <c r="C4" s="3">
         <v>30.0</v>
       </c>
-      <c r="C4" s="3">
+      <c r="D4" s="3">
         <v>0.0</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>6</v>
+      <c r="E4" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>